<commit_message>
Matrix builder: a logged bug counts as not reproduced only after a clean run of its journey
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/traceability-matrix.xlsx
+++ b/doc/traceability-matrix.xlsx
@@ -60839,14 +60839,10 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>j06-free-agent run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -60876,14 +60872,10 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>j07-team-application run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -60913,14 +60905,10 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>j07-team-application run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -60950,14 +60938,10 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr">
-        <is>
-          <t>j07-team-application run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -61024,14 +61008,10 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>j08-captain-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -61061,14 +61041,10 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>j06-free-agent run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -61098,14 +61074,10 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr">
-        <is>
-          <t>j06-free-agent run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -61135,14 +61107,10 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr">
-        <is>
-          <t>j08-captain-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -61209,14 +61177,10 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>j07-team-application run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -61246,14 +61210,10 @@
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>j08-captain-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -61283,14 +61243,10 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G16" t="inlineStr">
-        <is>
-          <t>j08-captain-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -61320,14 +61276,10 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G17" t="inlineStr">
-        <is>
-          <t>j08-captain-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -61357,14 +61309,10 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>j06-free-agent run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -61394,14 +61342,10 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G19" t="inlineStr">
-        <is>
-          <t>j08-captain-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -61431,14 +61375,10 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>j08-captain-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -61505,14 +61445,10 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>j07-team-application run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -61542,14 +61478,10 @@
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G23" t="inlineStr">
-        <is>
-          <t>j07-team-application run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -61579,14 +61511,10 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G24" t="inlineStr">
-        <is>
-          <t>j07-team-application run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -61616,14 +61544,10 @@
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G25" t="inlineStr">
-        <is>
-          <t>j08-captain-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -61690,14 +61614,10 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr">
-        <is>
-          <t>j09-eligibility run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -61764,14 +61684,10 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr">
-        <is>
-          <t>j09-eligibility run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -61801,14 +61717,10 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr">
-        <is>
-          <t>j09-eligibility run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -61838,14 +61750,10 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr">
-        <is>
-          <t>j09-eligibility run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -61875,14 +61783,10 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G32" t="inlineStr">
-        <is>
-          <t>j09-eligibility run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -61912,14 +61816,10 @@
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>j09-eligibility run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -61949,14 +61849,10 @@
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G34" t="inlineStr">
-        <is>
-          <t>j09-eligibility run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -61986,14 +61882,10 @@
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G35" t="inlineStr">
-        <is>
-          <t>j09-eligibility run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -62023,14 +61915,10 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -62060,14 +61948,10 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G37" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -62097,14 +61981,10 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -62134,14 +62014,10 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -62171,14 +62047,10 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -62208,14 +62080,10 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -62537,14 +62405,10 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G50" t="inlineStr">
-        <is>
-          <t>j04-player-registration run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -62574,14 +62438,10 @@
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G51" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -62611,14 +62471,10 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G52" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -62759,14 +62615,10 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -62796,14 +62648,10 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -62833,14 +62681,10 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G58" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -62907,14 +62751,10 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G60" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -62944,14 +62784,10 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -62981,14 +62817,10 @@
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G62" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -63018,14 +62850,10 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -63055,14 +62883,10 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -63092,14 +62916,10 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -63129,14 +62949,10 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G66" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -63166,14 +62982,10 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G67" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -63203,14 +63015,10 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G68" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -63277,14 +63085,10 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G70" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -63314,14 +63118,10 @@
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -63487,14 +63287,10 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G76" t="inlineStr">
-        <is>
-          <t>j04-player-registration run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -63561,14 +63357,10 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr">
-        <is>
-          <t>j04-player-registration run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -63672,14 +63464,10 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr">
-        <is>
-          <t>j04-player-registration run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -63783,14 +63571,10 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G84" t="inlineStr">
-        <is>
-          <t>j03-form run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -63820,14 +63604,10 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr">
-        <is>
-          <t>j03-form run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -63857,14 +63637,10 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>j03-form run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -63894,14 +63670,10 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr">
-        <is>
-          <t>j03-form run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -63931,14 +63703,10 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr">
-        <is>
-          <t>j05-minor-consent run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -63968,14 +63736,10 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr">
-        <is>
-          <t>j04-player-registration run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -64038,14 +63802,10 @@
       <c r="E91" t="inlineStr"/>
       <c r="F91" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G91" t="inlineStr">
-        <is>
-          <t>j03-form run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -64071,14 +63831,10 @@
       <c r="E92" t="inlineStr"/>
       <c r="F92" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G92" t="inlineStr">
-        <is>
-          <t>j03-form run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -64108,14 +63864,10 @@
       </c>
       <c r="F93" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G93" t="inlineStr">
-        <is>
-          <t>j03-form run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -64141,14 +63893,10 @@
       <c r="E94" t="inlineStr"/>
       <c r="F94" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G94" t="inlineStr">
-        <is>
-          <t>j04-player-registration run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -64174,14 +63922,10 @@
       <c r="E95" t="inlineStr"/>
       <c r="F95" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G95" t="inlineStr">
-        <is>
-          <t>j03-form run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -64207,14 +63951,10 @@
       <c r="E96" t="inlineStr"/>
       <c r="F96" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G96" t="inlineStr">
-        <is>
-          <t>j04-player-registration run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -64240,14 +63980,10 @@
       <c r="E97" t="inlineStr"/>
       <c r="F97" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G97" t="inlineStr">
-        <is>
-          <t>j05-minor-consent run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -64273,14 +64009,10 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr">
-        <is>
-          <t>j04-player-registration run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -64413,14 +64145,10 @@
       </c>
       <c r="F102" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G102" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -64450,14 +64178,10 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -64524,14 +64248,10 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -64561,14 +64281,10 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -64598,14 +64314,10 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -64635,14 +64347,10 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -64672,14 +64380,10 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -64709,14 +64413,10 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -64746,14 +64446,10 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G111" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -64783,14 +64479,10 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G112" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -64820,14 +64512,10 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -64857,14 +64545,10 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -64894,14 +64578,10 @@
       </c>
       <c r="F115" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G115" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -64931,14 +64611,10 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -64968,14 +64644,10 @@
       </c>
       <c r="F117" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G117" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -65005,14 +64677,10 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G118" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -65042,14 +64710,10 @@
       </c>
       <c r="F119" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G119" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -65079,14 +64743,10 @@
       </c>
       <c r="F120" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G120" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -65116,14 +64776,10 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G121" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G121" t="inlineStr"/>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -65153,14 +64809,10 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G122" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G122" t="inlineStr"/>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -65190,14 +64842,10 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G123" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G123" t="inlineStr"/>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -65449,14 +65097,10 @@
       </c>
       <c r="F130" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G130" t="inlineStr">
-        <is>
-          <t>j02-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G130" t="inlineStr"/>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -65486,14 +65130,10 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G131" t="inlineStr">
-        <is>
-          <t>j02-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G131" t="inlineStr"/>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -65597,14 +65237,10 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G134" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G134" t="inlineStr"/>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -65634,14 +65270,10 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G135" t="inlineStr">
-        <is>
-          <t>j02-invite run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G135" t="inlineStr"/>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -65745,14 +65377,10 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G138" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G138" t="inlineStr"/>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -65782,14 +65410,10 @@
       </c>
       <c r="F139" t="inlineStr">
         <is>
-          <t>not reproduced</t>
-        </is>
-      </c>
-      <c r="G139" t="inlineStr">
-        <is>
-          <t>j01-setup run on staging did not report it</t>
-        </is>
-      </c>
+          <t>open</t>
+        </is>
+      </c>
+      <c r="G139" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Matrix: record the scorekeeping, registration, money and placement fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/traceability-matrix.xlsx
+++ b/doc/traceability-matrix.xlsx
@@ -75839,10 +75839,14 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>commit 8333b60: people search and person reads limited to the caller's scope</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -75909,10 +75913,14 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>blockers-oct24-b (edit season incl. registration window) + status hints state the real rule</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -76453,10 +76461,14 @@
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G30" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>commit b3c8998: /compliance lists and signs required documents</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -77375,10 +77387,14 @@
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>not reproduced on branch (MON fix round 25 Oct)</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -77408,10 +77424,14 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G57" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>not reproduced on branch (MON fix round 25 Oct)</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -77552,10 +77572,14 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G61" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>commit 370cb34: RefundService caps refunds, lowers total+paid, idempotent</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -77622,10 +77646,14 @@
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>commit 370cb34 + migration 0053 (staging applied; production pending)</t>
+        </is>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -77688,10 +77716,14 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G65" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>commit 370cb34: compose targets org/league/season/division/team (schedule-later not built)</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -78133,10 +78165,14 @@
       </c>
       <c r="F78" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G78" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>commit b3c8998: pay/submit refused until required waivers signed</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -78240,10 +78276,14 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G81" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>commit b3c8998: active published form version bound and verified</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -78512,10 +78552,14 @@
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G89" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>commit b3c8998: window enforced before any write</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -78785,10 +78829,14 @@
       <c r="E98" t="inlineStr"/>
       <c r="F98" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G98" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>commit b3c8998: league forms only for that league's seasons</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -79024,10 +79072,14 @@
       </c>
       <c r="F105" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G105" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>commit a6bf6b5: scoped game access for league admins, scorekeepers, referees</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -79057,10 +79109,14 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G106" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>commit a6bf6b5: assists from the scoring team's roster</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -79090,10 +79146,14 @@
       </c>
       <c r="F107" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G107" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>commit a6bf6b5: infraction + minutes, PIM in stat lines</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -79123,10 +79183,14 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G108" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>commit a6bf6b5: finalize transaction projects stats + standings, notifies teams</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -79156,10 +79220,14 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G109" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>commit a6bf6b5: publish to team schedules</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -79189,10 +79257,14 @@
       </c>
       <c r="F110" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G110" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>commit a6bf6b5: reschedule with clash checks</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -79255,10 +79327,14 @@
       </c>
       <c r="F112" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G112" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>commit 4700c18: Add a team on the division page; j10 step 2 drives it</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -79391,10 +79467,14 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G116" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>commit a6bf6b5: captain /stats division table + player lines</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">

</xml_diff>

<commit_message>
Matrix: record the second fix wave
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/doc/traceability-matrix.xlsx
+++ b/doc/traceability-matrix.xlsx
@@ -75773,10 +75773,14 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>commit 200733b: claim is an offer the player accepts or declines</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -75806,10 +75810,14 @@
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>commit 200733b: admin free-agent pool panel with Assign to team</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -76358,10 +76366,14 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G27" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>commit 200733b: Documents to review queue with approve / reject / request new upload</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -76428,10 +76440,14 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G29" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>commit 200733b + migration 0054 (staging applied): player/guardian document upload</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -76498,10 +76514,14 @@
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G31" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>commit 200733b: sweeps never overwrite an admin waiver</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -76667,10 +76687,14 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G36" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>commit 200733b: issue / lift suspensions; served games counted at finalize</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -76733,10 +76757,14 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G38" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>commit 200733b: captain compliance lists suspended players</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -76766,10 +76794,14 @@
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>commit 200733b: lineup save refuses suspended starters/bench</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -76799,10 +76831,14 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>commit 200733b: sweep: missing data pending, suspension ineligible</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -78420,10 +78456,14 @@
       </c>
       <c r="F85" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G85" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>commit 200733b: player-app links from the API's PLAYER_WEB_URL</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -78453,10 +78493,14 @@
       </c>
       <c r="F86" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G86" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>commit 200733b: same as REG-12</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -78486,10 +78530,14 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G87" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>commit 200733b: registration type (team / individual / both) enforced</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -78519,10 +78567,14 @@
       </c>
       <c r="F88" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G88" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>commit 200733b: guardian consent records typed name, text, IP, browser</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -79002,10 +79054,14 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G103" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>commit 200733b: searchable, complete team pickers</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -79364,10 +79420,14 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G113" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>commit 200733b: New game picks season, division, entered teams, rink</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -79397,10 +79457,14 @@
       </c>
       <c r="F114" t="inlineStr">
         <is>
-          <t>open</t>
-        </is>
-      </c>
-      <c r="G114" t="inlineStr"/>
+          <t>fixed in code, not deployed</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>commit 200733b: rinks/surfaces editable, delete refused while in use, slots editable</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">

</xml_diff>